<commit_message>
Change mcu type select to be pull down for RX board
</commit_message>
<xml_diff>
--- a/pin_description.xlsx
+++ b/pin_description.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pig\Documents\GitHub\RC_Car\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACCA2055-276D-4A66-AF88-2CA7941196AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{576BB563-4789-4F4C-B912-35D79E6EB0B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2A8BD241-75E0-4CD8-AD8E-0F37EAB33EF2}"/>
   </bookViews>
@@ -253,21 +253,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -607,180 +604,179 @@
   <cols>
     <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" style="6"/>
     <col min="9" max="9" width="10" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="1" t="s">
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="2" t="s">
+      <c r="F3" s="1"/>
+      <c r="G3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>1</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="2">
         <v>1</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B5" s="9">
+      <c r="B5" s="5">
         <v>2</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="D5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="G5" s="9">
+      <c r="G5" s="5">
         <v>2</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="H5" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="I5" s="9" t="s">
+      <c r="I5" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="J5" s="9" t="s">
+      <c r="J5" s="5" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B6" s="7">
+      <c r="B6" s="3">
         <v>3</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="3">
         <v>3</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="I6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="J6" s="3" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B7" s="11">
+      <c r="B7" s="7">
         <v>4</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G7" s="11">
+      <c r="G7" s="7">
         <v>4</v>
       </c>
-      <c r="H7" s="11" t="s">
+      <c r="H7" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="I7" s="11" t="s">
+      <c r="I7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="J7" s="11" t="s">
+      <c r="J7" s="7" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B8" s="7">
+      <c r="B8" s="3">
         <v>5</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="4">
         <v>5</v>
       </c>
-      <c r="H8" s="8" t="s">
+      <c r="H8" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="I8" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="J8" s="8" t="s">
+      <c r="J8" s="4" t="s">
         <v>42</v>
       </c>
     </row>
@@ -837,16 +833,16 @@
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B12" s="8">
+      <c r="B12" s="4">
         <v>8</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="D12" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="4" t="s">
         <v>43</v>
       </c>
       <c r="G12">
@@ -863,80 +859,80 @@
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B13" s="7">
+      <c r="B13" s="3">
         <v>9</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="G13" s="7">
+      <c r="G13" s="3">
         <v>9</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="H13" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I13" s="7" t="s">
+      <c r="I13" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="J13" s="7" t="s">
+      <c r="J13" s="3" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B14" s="7">
+      <c r="B14" s="3">
         <v>10</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="G14" s="7">
+      <c r="G14" s="3">
         <v>10</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="H14" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="I14" s="7" t="s">
+      <c r="I14" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="J14" s="7" t="s">
+      <c r="J14" s="3" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B15" s="8">
+      <c r="B15" s="4">
         <v>11</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="G15" s="7">
+      <c r="G15" s="3">
         <v>11</v>
       </c>
-      <c r="H15" s="7" t="s">
+      <c r="H15" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I15" s="7" t="s">
+      <c r="I15" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="J15" s="7" t="s">
+      <c r="J15" s="3" t="s">
         <v>41</v>
       </c>
     </row>
@@ -953,68 +949,68 @@
       <c r="E16" t="s">
         <v>40</v>
       </c>
-      <c r="G16" s="8">
+      <c r="G16" s="4">
         <v>12</v>
       </c>
-      <c r="H16" s="8" t="s">
+      <c r="H16" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="I16" s="8" t="s">
+      <c r="I16" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="J16" s="8" t="s">
+      <c r="J16" s="4" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B17" s="10">
+      <c r="B17" s="6">
         <v>13</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="E17" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="G17" s="10">
+      <c r="G17" s="6">
         <v>13</v>
       </c>
-      <c r="H17" s="10" t="s">
+      <c r="H17" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="I17" s="10" t="s">
+      <c r="I17" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="J17" s="10" t="s">
+      <c r="J17" s="6" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B18" s="3">
+      <c r="B18" s="2">
         <v>14</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E18" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="G18" s="3">
+      <c r="G18" s="2">
         <v>14</v>
       </c>
-      <c r="H18" s="3" t="s">
+      <c r="H18" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I18" s="3" t="s">
+      <c r="I18" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="J18" s="3" t="s">
+      <c r="J18" s="2" t="s">
         <v>44</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Working motor and servo driver code
</commit_message>
<xml_diff>
--- a/pin_description.xlsx
+++ b/pin_description.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pig\Documents\GitHub\RC_Car\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6916CF7B-AD3A-4057-B8F6-6781F993E13A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D2A71D7-FD96-4594-AE62-8F448237CA85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2A8BD241-75E0-4CD8-AD8E-0F37EAB33EF2}"/>
+    <workbookView xWindow="735" yWindow="675" windowWidth="13800" windowHeight="11325" xr2:uid="{2A8BD241-75E0-4CD8-AD8E-0F37EAB33EF2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="47">
   <si>
     <t>Vdd</t>
   </si>
@@ -174,6 +174,9 @@
   </si>
   <si>
     <t>program/NC</t>
+  </si>
+  <si>
+    <t>RC4</t>
   </si>
 </sst>
 </file>
@@ -785,7 +788,7 @@
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="D9" t="s">
         <v>21</v>
@@ -797,7 +800,7 @@
         <v>6</v>
       </c>
       <c r="H9" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
       <c r="I9" t="s">
         <v>31</v>

</xml_diff>